<commit_message>
Add patient and office columns to Slip Activity Monitor
RXN-9 scope addition: show patient_name and office_name (provisional
backend field names) in the table, fixtures, tests and i18n.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/e2e/fixtures/slip-activity/export.xlsx
+++ b/e2e/fixtures/slip-activity/export.xlsx
@@ -23,15 +23,25 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>From status</t>
+          <t>Patient</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>From status</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>To status</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>User</t>
         </is>
@@ -50,15 +60,25 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>In lab</t>
+          <t>John Doe</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>Smile Dental</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>In lab</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>In lab ready to pickup</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Maria Lopez</t>
         </is>

</xml_diff>

<commit_message>
Match Slip Activity office field to backend contract
RXN-9: events rows carry office as { id, name } or null (not office_name);
export adds Patient name and Office at the end. Update types, row mapping,
tests and mock fixtures.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/e2e/fixtures/slip-activity/export.xlsx
+++ b/e2e/fixtures/slip-activity/export.xlsx
@@ -23,27 +23,27 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Patient</t>
+          <t>From status</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>To status</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>From status</t>
+          <t>User</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>To status</t>
+          <t>Patient name</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>User</t>
+          <t>Office</t>
         </is>
       </c>
     </row>
@@ -60,27 +60,27 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>John Doe</t>
+          <t>In lab</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Smile Dental</t>
+          <t>In lab ready to pickup</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>In lab</t>
+          <t>Maria Lopez</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>In lab ready to pickup</t>
+          <t>John Doe</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Maria Lopez</t>
+          <t>Smile Dental</t>
         </is>
       </c>
     </row>

</xml_diff>